<commit_message>
sprint plan backlog for sprint 3
</commit_message>
<xml_diff>
--- a/BusinessAnalysis/ProductBacklog.xlsx
+++ b/BusinessAnalysis/ProductBacklog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Micro2Move\BusinessAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7042DDE-F20C-4EEB-87A5-034AFD03859A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8361249-CAAB-418D-8615-1E6359747304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="13044" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProductBacklog" sheetId="1" r:id="rId1"/>
@@ -3810,9 +3810,6 @@
     </r>
   </si>
   <si>
-    <t>I can see all the commnity updates</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">I must be able to see community updates (if any) screen, with </t>
     </r>
@@ -5604,6 +5601,9 @@
       <t xml:space="preserve"> sorted in ascending order of price.
 2. I must be able to see if the E-Bike is platform verified or not, signified by the presence of a verified badge.</t>
     </r>
+  </si>
+  <si>
+    <t>I can see all the community updates</t>
   </si>
 </sst>
 </file>
@@ -6510,7 +6510,7 @@
       <c r="A17" s="7"/>
       <c r="B17" s="1"/>
       <c r="C17" s="10" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>15</v>
@@ -6746,7 +6746,7 @@
         <v>70</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H29" s="12" t="s">
         <v>66</v>
@@ -6760,7 +6760,7 @@
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
       <c r="G30" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H30" s="4"/>
     </row>
@@ -6978,7 +6978,7 @@
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H44" s="12"/>
     </row>
@@ -7002,7 +7002,7 @@
         <v>95</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H45" s="14" t="s">
         <v>43</v>
@@ -7019,7 +7019,7 @@
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
       <c r="G46" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H46" s="5"/>
     </row>
@@ -7031,7 +7031,7 @@
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
       <c r="G47" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H47" s="14" t="s">
         <v>97</v>
@@ -7045,7 +7045,7 @@
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H48" s="14"/>
     </row>
@@ -7059,7 +7059,7 @@
         <v>3</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F49" s="5" t="s">
         <v>98</v>
@@ -7107,7 +7107,7 @@
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
       <c r="G51" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H51" s="5"/>
     </row>
@@ -7192,16 +7192,16 @@
         <v>3.6</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E56" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="F56" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="F56" s="5" t="s">
-        <v>195</v>
-      </c>
       <c r="G56" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H56" s="14" t="s">
         <v>94</v>
@@ -7217,19 +7217,19 @@
         <v>3.7</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E57" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="G57" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="F57" s="5" t="s">
+      <c r="H57" s="14" t="s">
         <v>196</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="H57" s="14" t="s">
-        <v>197</v>
       </c>
       <c r="I57" s="14" t="s">
         <v>43</v>
@@ -7242,19 +7242,19 @@
         <v>3.8</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E58" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="F58" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="F58" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="G58" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H58" s="14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="59" spans="1:10" ht="216" x14ac:dyDescent="0.3">
@@ -7267,100 +7267,100 @@
         <v>3</v>
       </c>
       <c r="E59" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G59" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="5" t="s">
+      <c r="H59" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="G59" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="H59" s="14" t="s">
-        <v>200</v>
-      </c>
       <c r="I59" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A60" s="13"/>
       <c r="B60" s="5"/>
       <c r="C60" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="H60" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="I60" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J60" s="14" t="s">
         <v>201</v>
-      </c>
-      <c r="D60" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="E60" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="H60" s="14" t="s">
-        <v>231</v>
-      </c>
-      <c r="I60" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="J60" s="14" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="288" x14ac:dyDescent="0.3">
       <c r="A61" s="13"/>
       <c r="B61" s="5"/>
       <c r="C61" s="25" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D61" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="F61" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G61" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="H61" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="F61" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="H61" s="14" t="s">
+      <c r="I61" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="I61" s="14" t="s">
+      <c r="J61" s="14" t="s">
         <v>208</v>
-      </c>
-      <c r="J61" s="14" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="148.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="13"/>
       <c r="B62" s="5"/>
       <c r="C62" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F62" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="D62" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="E62" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F62" s="5" t="s">
+      <c r="G62" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="H62" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="I62" s="14" t="s">
         <v>211</v>
-      </c>
-      <c r="G62" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="H62" s="14" t="s">
-        <v>207</v>
-      </c>
-      <c r="I62" s="14" t="s">
-        <v>212</v>
       </c>
       <c r="J62" s="27"/>
     </row>
@@ -7368,19 +7368,19 @@
       <c r="A63" s="13"/>
       <c r="B63" s="5"/>
       <c r="C63" s="25" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E63" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F63" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="G63" s="5" t="s">
         <v>227</v>
-      </c>
-      <c r="F63" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="G63" s="5" t="s">
-        <v>228</v>
       </c>
       <c r="H63" s="27"/>
       <c r="I63" s="27"/>
@@ -7492,13 +7492,13 @@
         <v>158</v>
       </c>
       <c r="F69" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="G69" s="19" t="s">
         <v>160</v>
       </c>
-      <c r="G69" s="19" t="s">
+      <c r="H69" s="21" t="s">
         <v>161</v>
-      </c>
-      <c r="H69" s="21" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="57.6" x14ac:dyDescent="0.3">
@@ -7514,13 +7514,13 @@
         <v>159</v>
       </c>
       <c r="F70" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="G70" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="G70" s="19" t="s">
+      <c r="H70" s="21" t="s">
         <v>164</v>
-      </c>
-      <c r="H70" s="21" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
@@ -7528,7 +7528,7 @@
         <v>5</v>
       </c>
       <c r="B71" s="23" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C71" s="22">
         <v>5.0999999999999996</v>
@@ -7537,16 +7537,16 @@
         <v>143</v>
       </c>
       <c r="E71" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="F71" s="23" t="s">
         <v>167</v>
       </c>
-      <c r="F71" s="23" t="s">
+      <c r="G71" s="23" t="s">
         <v>168</v>
       </c>
-      <c r="G71" s="23" t="s">
+      <c r="H71" s="24" t="s">
         <v>169</v>
-      </c>
-      <c r="H71" s="24" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -7559,16 +7559,16 @@
         <v>143</v>
       </c>
       <c r="E72" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="F72" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="F72" s="23" t="s">
+      <c r="G72" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="G72" s="23" t="s">
+      <c r="H72" s="24" t="s">
         <v>173</v>
-      </c>
-      <c r="H72" s="24" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -7581,16 +7581,16 @@
         <v>143</v>
       </c>
       <c r="E73" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="F73" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="F73" s="23" t="s">
+      <c r="G73" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="G73" s="23" t="s">
+      <c r="H73" s="24" t="s">
         <v>177</v>
-      </c>
-      <c r="H73" s="24" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
@@ -7603,13 +7603,13 @@
         <v>143</v>
       </c>
       <c r="E74" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="F74" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="F74" s="23" t="s">
+      <c r="G74" s="23" t="s">
         <v>180</v>
-      </c>
-      <c r="G74" s="23" t="s">
-        <v>181</v>
       </c>
       <c r="H74" s="23"/>
     </row>

</xml_diff>

<commit_message>
Supplier Auth, Fleet management added
</commit_message>
<xml_diff>
--- a/BusinessAnalysis/ProductBacklog.xlsx
+++ b/BusinessAnalysis/ProductBacklog.xlsx
@@ -1,37 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Micro2Move\BusinessAnalysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ANODIAM\Micro2Move\BusinessAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8361249-CAAB-418D-8615-1E6359747304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B62B51B9-E1AF-48B3-862B-DC43C37F092F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="13044" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProductBacklog" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="264">
   <si>
     <t>As a</t>
   </si>
@@ -5604,13 +5593,135 @@
   </si>
   <si>
     <t>I can see all the community updates</t>
+  </si>
+  <si>
+    <t>Supplier Auth</t>
+  </si>
+  <si>
+    <t>Unregistered Product Owner</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">I want to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>attempt to log in using my email and password</t>
+    </r>
+  </si>
+  <si>
+    <t>I can access the Supplier Portal</t>
+  </si>
+  <si>
+    <t>If I enter an email that is not registered in the system, I must see an error message: “Account not found. Please register to continue.” I must be given a clear Register button / hyperlink.</t>
+  </si>
+  <si>
+    <t>I can request access to the Supplier Portal</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">I want to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>register my business details</t>
+    </r>
+  </si>
+  <si>
+    <t>I must be able to enter Store Name, Location, ABN, Email, Password, Owner/Manager Name and Phone Number. All fields must be mandatory. If any field is invalid, respective error messages must be shown on the same screen. If all details are valid, I must see a success message: “Thank you for registering! Admin will soon grant you access.”</t>
+  </si>
+  <si>
+    <t>If I enter valid credentials and my account status is Approved, I must be successfully logged in. If I have no existing fleet listings, I must be redirected to the “List Your First e-Bike Fleet” screen. The screen must display a large “+” button to add my first fleet. A welcome header must be visible.</t>
+  </si>
+  <si>
+    <t>Approved Product Owner with Existing Fleets</t>
+  </si>
+  <si>
+    <t>I want to log in using valid credentials</t>
+  </si>
+  <si>
+    <t>I can manage my existing e-bike fleets</t>
+  </si>
+  <si>
+    <t>If I enter valid credentials and I already have one or more fleets listed, I must be redirected to the “Your e-Bike Fleets” screen. I must see all my listed fleets with: Fleet Name, Image, Price per week, Category, Location and Quantity (Qty). I must see a “List Another Fleet” button at the bottom.</t>
+  </si>
+  <si>
+    <t>Fleet Management</t>
+  </si>
+  <si>
+    <t>Approved Product Owner (No Existing Fleets)</t>
+  </si>
+  <si>
+    <t>I want to add my first e-Bike fleet</t>
+  </si>
+  <si>
+    <t>I can make my bikes available for rental on Micro2Move</t>
+  </si>
+  <si>
+    <t>If I am a logged-in and approved Product Owner with no existing fleets, I must be redirected to the “List Your First e-Bike Fleet” screen. I must see a large “+” button to add my first fleet. When I press the “+” button, I must be navigated to the e-Bike Fleet creation form.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved Product Owner </t>
+  </si>
+  <si>
+    <t>I want to open the side menu from the fleet screen</t>
+  </si>
+  <si>
+    <t>I can navigate to Manage Listing, Analytics, or Profile</t>
+  </si>
+  <si>
+    <t>If I tap on the three-dot menu icon from the Fleet screen, I must see a side menu panel open. The side menu must display the following options:1.ManageListing 2.Analytics 3.Profile. A close (X) icon must be visible at the top right corner. If I tap the close (X) icon, the menu must close and return to the previous screen.</t>
+  </si>
+  <si>
+    <t>I want to select “Manage Listing” from the side menu</t>
+  </si>
+  <si>
+    <t>If I tap on “Manage Listing”, I must be redirected to the Manage Listing screen.
+The Manage Listing option must be visually highlighted when selected.</t>
+  </si>
+  <si>
+    <t>I want to select “Analytics” from the side menu</t>
+  </si>
+  <si>
+    <t>I can view my fleet performance insights</t>
+  </si>
+  <si>
+    <t>I can edit or manage my fleet details</t>
+  </si>
+  <si>
+    <t>If I tap on “Analytics”, I must be redirected to the Analytics dashboard screen.
+The Analytics option must be visually highlighted when selected.</t>
+  </si>
+  <si>
+    <t>I want to select “Profile” from the side menu</t>
+  </si>
+  <si>
+    <t>I can view and manage my supplier profile</t>
+  </si>
+  <si>
+    <t>If I tap on “Profile”, I must be redirected to the Supplier Profile screen.
+The Profile option must be visually highlighted when selected</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5648,8 +5759,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5716,6 +5834,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -5771,7 +5901,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -5859,6 +5989,42 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6150,13 +6316,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K74"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.109375" style="9" customWidth="1"/>
     <col min="2" max="2" width="11.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="6.33203125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="24" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24.77734375" style="2" customWidth="1"/>
     <col min="7" max="7" width="40.44140625" style="2" customWidth="1"/>
@@ -7594,24 +7760,185 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A74" s="22"/>
-      <c r="B74" s="23"/>
-      <c r="C74" s="22">
+      <c r="A74" s="37"/>
+      <c r="B74" s="38"/>
+      <c r="C74" s="37">
         <v>5.4</v>
       </c>
-      <c r="D74" s="23" t="s">
+      <c r="D74" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="E74" s="23" t="s">
+      <c r="E74" s="38" t="s">
         <v>178</v>
       </c>
-      <c r="F74" s="23" t="s">
+      <c r="F74" s="38" t="s">
         <v>179</v>
       </c>
-      <c r="G74" s="23" t="s">
+      <c r="G74" s="38" t="s">
         <v>180</v>
       </c>
-      <c r="H74" s="23"/>
+      <c r="H74" s="38"/>
+    </row>
+    <row r="75" spans="1:9" s="36" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="35"/>
+      <c r="C75" s="35"/>
+    </row>
+    <row r="76" spans="1:9" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="39">
+        <v>6</v>
+      </c>
+      <c r="B76" s="40" t="s">
+        <v>233</v>
+      </c>
+      <c r="C76" s="39">
+        <v>6.1</v>
+      </c>
+      <c r="D76" s="40" t="s">
+        <v>234</v>
+      </c>
+      <c r="E76" s="41" t="s">
+        <v>235</v>
+      </c>
+      <c r="F76" s="41" t="s">
+        <v>236</v>
+      </c>
+      <c r="G76" s="40" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A77" s="30"/>
+      <c r="B77" s="31"/>
+      <c r="C77" s="30">
+        <v>6.2</v>
+      </c>
+      <c r="D77" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="E77" s="31" t="s">
+        <v>239</v>
+      </c>
+      <c r="F77" s="31" t="s">
+        <v>238</v>
+      </c>
+      <c r="G77" s="31" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A78" s="30"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="30"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="31"/>
+      <c r="F78" s="31"/>
+      <c r="G78" s="31" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="89.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="32">
+        <v>7</v>
+      </c>
+      <c r="B79" s="33" t="s">
+        <v>246</v>
+      </c>
+      <c r="C79" s="32">
+        <v>7.1</v>
+      </c>
+      <c r="D79" s="33" t="s">
+        <v>247</v>
+      </c>
+      <c r="E79" s="33" t="s">
+        <v>248</v>
+      </c>
+      <c r="F79" s="33" t="s">
+        <v>249</v>
+      </c>
+      <c r="G79" s="34" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A80" s="32"/>
+      <c r="B80" s="34"/>
+      <c r="C80" s="32"/>
+      <c r="D80" s="33" t="s">
+        <v>242</v>
+      </c>
+      <c r="E80" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="F80" s="33" t="s">
+        <v>244</v>
+      </c>
+      <c r="G80" s="34" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="105" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="32"/>
+      <c r="B81" s="34"/>
+      <c r="C81" s="32">
+        <v>7.2</v>
+      </c>
+      <c r="D81" s="34" t="s">
+        <v>251</v>
+      </c>
+      <c r="E81" s="33" t="s">
+        <v>252</v>
+      </c>
+      <c r="F81" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="G81" s="34" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A82" s="32"/>
+      <c r="B82" s="34"/>
+      <c r="C82" s="32"/>
+      <c r="D82" s="34"/>
+      <c r="E82" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="F82" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="G82" s="34" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A83" s="32"/>
+      <c r="B83" s="34"/>
+      <c r="C83" s="32"/>
+      <c r="D83" s="34"/>
+      <c r="E83" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="F83" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="G83" s="34" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A84" s="32"/>
+      <c r="B84" s="34"/>
+      <c r="C84" s="32"/>
+      <c r="D84" s="34"/>
+      <c r="E84" s="34" t="s">
+        <v>261</v>
+      </c>
+      <c r="F84" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="G84" s="34" t="s">
+        <v>263</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>